<commit_message>
docs: adiciona a versão 8 do artigo e atualiza as referências
- corrige números (percentis do preço, FRAME, P210, MGTe Elite, TOTAL_SELOS)
- descreve a validação aninhada, a significância marginal do MATERNAL e a regra
  das linhagens; ajusta citações de Carneiro Junior, Braga, Silveira, Pacheco e Breiman
- inclui Spence (1973) e Gomes (2019), nova Figura 2, fonte nas tabelas e
  formatação ABNT das referências
- planilha de verificação com a aba Atualizacao_v8
</commit_message>
<xml_diff>
--- a/Referencias/Verificacao_citacoes.xlsx
+++ b/Referencias/Verificacao_citacoes.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discussao" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referencias_ABNT" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problemas_rascunho" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atualizacao_v8" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4783,4 +4784,478 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Onde no texto (v8)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Afirmação no texto</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Citação</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Arquivo local</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Link / DOI</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Página no PDF</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Trecho literal da fonte</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Alteração no v8</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Conferido? (S/N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Selos – parágrafo do Akerlof</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Os selos aproximam-se dos sinais de mercado descritos por Spence: atributos observáveis a partir dos quais o comprador infere características que não consegue verificar diretamente</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>SPENCE, 1973</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Spence_1973_QJE.pdf</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2307/1882010</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2 (p. 356 da revista)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>PDF escaneado: conferir na imagem da p. 356 a definição de signals (observable, alterable characteristics)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Nova citação: dá base à "sinalização comercial" do resumo e da conclusão</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Selos – parágrafo do Akerlof</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>O grande número de DEPs, acurácias e percentis tende a dificultar a tomada de decisão na seleção</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GOMES, 2019</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Gomes_2019_UFMS.pdf</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>"O aprimoramento das técnicas de avaliação genética tem gerado número cada vez maior de informações, disponibilizando DEPs para diferentes características, o que tem dificultado os processos de tomada de decisão na seleção."</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Nova citação: a frase estava sem fonte (Gomes cita Tonhati et al., 2003)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Selos – parágrafo do Akerlof</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Em leilões, parte dos compradores privilegia a apresentação visual do animal em relação às informações técnicas</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>SILVEIRA, 2022</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Silveira_2022_UFMS.pdf</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>"Do outro lado da régua, encontra-se o comprador mais visual. Neste caso, o animal bem apresentado visualmente tem vantagem"</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Reescrita: "visual" é a aparência do animal no leilão, não um selo gráfico</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Linhagens</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>O leiloeiro entrevistado apontou a marca como o principal agregador de valor</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SILVEIRA, 2022</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Silveira_2022_UFMS.pdf</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>"Ao final da entrevista com o leiloeiro, este apontou que a marca, na opinião dele, é o principal agregador de valor"</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Reescrita: a fonte diz "a marca", não "a marca do criatório"</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Carcaça (AOL/ACAB)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Frigoríficos bonificam pela espessura de gordura (3 a 6 mm); abaixo de 3 mm, carne menos macia, com efeito marginal na meta-análise</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>PACHECO et al., 2023</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Pacheco_2023_PAB.pdf</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1590/S1678-3921.pab2023.v58.03110</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1 e 5</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>"Carcasses with a fat thickness less than 3 mm produce tougher meat" (resumo); "The shear force increased (p=0.0835)" (p. 5)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Suavizada: "segundo a revisão de Pacheco et al."; efeito marginal explicitado</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>DEPs – regressão</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>P450, STAY e P210 respondem por cerca de 62% do MGTe, segundo a ponderação da ANCP de 2021</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>SILVEIRA, 2022</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Silveira_2022_UFMS.pdf</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>"formam aproximadamente 62% do índice proposto como MGTe" (Quadro 06, fonte ANCP 2021)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Acrescentado "segundo a ponderação da ANCP de 2021"</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Métodos – variáveis</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>18 DEPs agrupadas, em sua maioria, conforme a ANCP; grupo "Produtividade e Qualidade da Carne"</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>SILVEIRA, 2022</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Silveira_2022_UFMS.pdf</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>70-72</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Quadro 05: grupos da ANCP</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Nome do grupo corrigido; FPP e FRAME indicados como do catálogo</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Discussão final</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Brangus no RS (Lopes); Nelore no Centro-Oeste, correlação com índice genético em 23% dos leilões (Carneiro Jr.); mesma base de dados (Braga)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>LOPES et al., 2023; CARNEIRO JUNIOR et al., 2024; BRAGA et al., 2023</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/CarneiroJunior_Embrapa_27753.pdf; Referencias/Braga_Embrapa_27547.pdf</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2-3 (Carneiro Jr.); 1 (Braga)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>"2.393 observações de touros da raça Nelore [...] em 62 leilões"; "23% foram classificados no grupo 1"</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Corrigido: as duas fontes Embrapa são de touros Nelore (Campo Grande), não Brangus, e usam a mesma base</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Métodos – Random Forest</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Descrição do algoritmo (bootstrap e sorteio de variáveis em cada divisão)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>BREIMAN, 2001</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/Breiman_2001_ML.pdf</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1023/A:1010933404324</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Random forests: bagging + random feature selection</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Retirada a justificativa "por acomodar relações não lineares e variáveis correlacionadas", que não está em Breiman; MDI atribuída ao scikit-learn</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Citação RP-ANCP</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>(REPRODUÇÃO [...], 2025)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>REPRODUÇÃO [...], 2025</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Referencias/paginas_web/OPresenteRural_2025_ANCP_Reproducao_Programada.html</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Supressão no título com [...] (NBR 10520:2023)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: corrige o resumo e a leitura da validação aninhada na versão 8 e retira Gomes (2019)
- resumo reduzido de 320 para 299 palavras (limite do template: 300)
- validação aninhada descrita como pouco melhor que o modelo sem preditores
  (R² -5,2% contra -10,4%; RMSE R$ 6,47 contra R$ 6,72), como mostra a Tabela 5;
  o texto dizia 'sem ganho sobre a média do preço'
- Gomes (2019) retirado do artigo (fonte com mais de 5 anos) e devolvido a
  Referencias/nao_citadas_no_artigo; índice e planilha de verificação atualizados
- PDF da versão 8
</commit_message>
<xml_diff>
--- a/Referencias/Verificacao_citacoes.xlsx
+++ b/Referencias/Verificacao_citacoes.xlsx
@@ -4914,7 +4914,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Referencias/Gomes_2019_UFMS.pdf</t>
+          <t>Referencias/nao_citadas_no_artigo/Gomes_2019_UFMS.pdf</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -4930,7 +4930,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Nova citação: a frase estava sem fonte (Gomes cita Tonhati et al., 2003)</t>
+          <t>RETIRADA em 15/10/2026 a pedido do autor (fonte com mais de 5 anos); a frase voltou a terminar em "apresentados para cada touro.", sem citação</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
docs: remonta a versão 8 do artigo pelo pipeline das partes e retira Spence (1973)
- o conteúdo da v8 feita na nuvem foi levado para as partes do artigo e o texto
  foi remontado com as regras de formatação de sempre (sem os itálicos, o negrito
  das referências e a fonte sob as tabelas que a nuvem acrescentou)
- Spence (1973) retirado: a teoria exige sinal custoso, que os selos concedidos
  pela central não têm, e o Akerlof já sustenta o argumento; PDF e texto voltam
  para Referencias/nao_citadas_no_artigo, com índice e planilha atualizados
- Figura 1 com 13,5 cm e Figura 4 antes da Tabela 5, para não deixar meia página
  em branco; figura, legenda e fonte na mesma página
</commit_message>
<xml_diff>
--- a/Referencias/Verificacao_citacoes.xlsx
+++ b/Referencias/Verificacao_citacoes.xlsx
@@ -4871,7 +4871,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Referencias/Spence_1973_QJE.pdf</t>
+          <t>Referencias/nao_citadas_no_artigo/Spence_1973_QJE.pdf</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -4881,20 +4881,24 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2 (p. 356 da revista)</t>
+          <t>4 (p. 357 da revista)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>PDF escaneado: conferir na imagem da p. 356 a definição de signals (observable, alterable characteristics)</t>
+          <t>Definição na p. 357: sinais são atributos observáveis alteráveis por quem os apresenta; os inalteráveis são índices</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Nova citação: dá base à "sinalização comercial" do resumo e da conclusão</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
+          <t>RETIRADA em 15/10/2026: a teoria exige sinal custoso, que os selos concedidos pela central não têm; o Akerlof já sustenta o argumento. A frase voltou a ser como na v7</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>